<commit_message>
Equilíbrio sustentado (50/30/27) no modelo, plano e deck
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PinPBG7GFUc6Efs6ijKbpo
</commit_message>
<xml_diff>
--- a/03_plano/Jalecon_Modelo_Financeiro.xlsx
+++ b/03_plano/Jalecon_Modelo_Financeiro.xlsx
@@ -470,7 +470,7 @@
     <t xml:space="preserve">EBITDA do ano 5 (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Primeiro mês com EBITDA positivo</t>
+    <t xml:space="preserve">Mês do equilíbrio (EBITDA positivo daí em diante)</t>
   </si>
   <si>
     <t xml:space="preserve">Menor saldo de caixa no período (R$)</t>
@@ -479,7 +479,7 @@
     <t xml:space="preserve">Total captado no período (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Leitura: 999 em 'primeiro mês com EBITDA positivo' significa que o cenário não chega ao equilíbrio em 60 meses. Caixa negativo indica necessidade de captação adicional.</t>
+    <t xml:space="preserve">Leitura: 999 em 'mês do equilíbrio' significa que o cenário não chega ao equilíbrio em 60 meses. Caixa negativo indica necessidade de captação adicional.</t>
   </si>
   <si>
     <t xml:space="preserve">Necessidade de caixa antes da rodada seed (cenário base)</t>
@@ -821,7 +821,7 @@
     <t xml:space="preserve">Churn mensal total (% da base do mês anterior)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mês com EBITDA positivo (auxiliar)</t>
+    <t xml:space="preserve">Mês com EBITDA positivo daí em diante (auxiliar)</t>
   </si>
   <si>
     <t xml:space="preserve">Jalecon: projeção mensal, cenário base</t>
@@ -1621,11 +1621,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="44452059"/>
-        <c:axId val="67386951"/>
+        <c:axId val="64965204"/>
+        <c:axId val="24614974"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="44452059"/>
+        <c:axId val="64965204"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1657,7 +1657,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67386951"/>
+        <c:crossAx val="24614974"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1665,7 +1665,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67386951"/>
+        <c:axId val="24614974"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1741,7 +1741,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44452059"/>
+        <c:crossAx val="64965204"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2032,11 +2032,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="88133499"/>
-        <c:axId val="85643894"/>
+        <c:axId val="24896822"/>
+        <c:axId val="11290059"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="88133499"/>
+        <c:axId val="24896822"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2068,7 +2068,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85643894"/>
+        <c:crossAx val="11290059"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2076,7 +2076,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85643894"/>
+        <c:axId val="11290059"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2118,7 +2118,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88133499"/>
+        <c:crossAx val="24896822"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B33" s="20" t="n">
         <f aca="false">MIN(Modelo_Conservador!$C$65:$BJ$65)</f>
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C33" s="20" t="n">
         <f aca="false">MIN(Modelo_Base!$C$65:$BJ$65)</f>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="D33" s="20" t="n">
         <f aca="false">MIN(Modelo_Otimista!$C$65:$BJ$65)</f>
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18522,243 +18522,243 @@
         <v>264</v>
       </c>
       <c r="C65" s="19" t="n">
-        <f aca="false">IF(C56&gt;0,C$3,999)</f>
+        <f aca="false">IF(MIN(C56:$BJ56)&gt;0,C$3,999)</f>
         <v>999</v>
       </c>
       <c r="D65" s="19" t="n">
-        <f aca="false">IF(D56&gt;0,D$3,999)</f>
+        <f aca="false">IF(MIN(D56:$BJ56)&gt;0,D$3,999)</f>
         <v>999</v>
       </c>
       <c r="E65" s="19" t="n">
-        <f aca="false">IF(E56&gt;0,E$3,999)</f>
+        <f aca="false">IF(MIN(E56:$BJ56)&gt;0,E$3,999)</f>
         <v>999</v>
       </c>
       <c r="F65" s="19" t="n">
-        <f aca="false">IF(F56&gt;0,F$3,999)</f>
+        <f aca="false">IF(MIN(F56:$BJ56)&gt;0,F$3,999)</f>
         <v>999</v>
       </c>
       <c r="G65" s="19" t="n">
-        <f aca="false">IF(G56&gt;0,G$3,999)</f>
+        <f aca="false">IF(MIN(G56:$BJ56)&gt;0,G$3,999)</f>
         <v>999</v>
       </c>
       <c r="H65" s="19" t="n">
-        <f aca="false">IF(H56&gt;0,H$3,999)</f>
+        <f aca="false">IF(MIN(H56:$BJ56)&gt;0,H$3,999)</f>
         <v>999</v>
       </c>
       <c r="I65" s="19" t="n">
-        <f aca="false">IF(I56&gt;0,I$3,999)</f>
+        <f aca="false">IF(MIN(I56:$BJ56)&gt;0,I$3,999)</f>
         <v>999</v>
       </c>
       <c r="J65" s="19" t="n">
-        <f aca="false">IF(J56&gt;0,J$3,999)</f>
+        <f aca="false">IF(MIN(J56:$BJ56)&gt;0,J$3,999)</f>
         <v>999</v>
       </c>
       <c r="K65" s="19" t="n">
-        <f aca="false">IF(K56&gt;0,K$3,999)</f>
+        <f aca="false">IF(MIN(K56:$BJ56)&gt;0,K$3,999)</f>
         <v>999</v>
       </c>
       <c r="L65" s="19" t="n">
-        <f aca="false">IF(L56&gt;0,L$3,999)</f>
+        <f aca="false">IF(MIN(L56:$BJ56)&gt;0,L$3,999)</f>
         <v>999</v>
       </c>
       <c r="M65" s="19" t="n">
-        <f aca="false">IF(M56&gt;0,M$3,999)</f>
+        <f aca="false">IF(MIN(M56:$BJ56)&gt;0,M$3,999)</f>
         <v>999</v>
       </c>
       <c r="N65" s="19" t="n">
-        <f aca="false">IF(N56&gt;0,N$3,999)</f>
+        <f aca="false">IF(MIN(N56:$BJ56)&gt;0,N$3,999)</f>
         <v>999</v>
       </c>
       <c r="O65" s="19" t="n">
-        <f aca="false">IF(O56&gt;0,O$3,999)</f>
+        <f aca="false">IF(MIN(O56:$BJ56)&gt;0,O$3,999)</f>
         <v>999</v>
       </c>
       <c r="P65" s="19" t="n">
-        <f aca="false">IF(P56&gt;0,P$3,999)</f>
+        <f aca="false">IF(MIN(P56:$BJ56)&gt;0,P$3,999)</f>
         <v>999</v>
       </c>
       <c r="Q65" s="19" t="n">
-        <f aca="false">IF(Q56&gt;0,Q$3,999)</f>
+        <f aca="false">IF(MIN(Q56:$BJ56)&gt;0,Q$3,999)</f>
         <v>999</v>
       </c>
       <c r="R65" s="19" t="n">
-        <f aca="false">IF(R56&gt;0,R$3,999)</f>
+        <f aca="false">IF(MIN(R56:$BJ56)&gt;0,R$3,999)</f>
         <v>999</v>
       </c>
       <c r="S65" s="19" t="n">
-        <f aca="false">IF(S56&gt;0,S$3,999)</f>
+        <f aca="false">IF(MIN(S56:$BJ56)&gt;0,S$3,999)</f>
         <v>999</v>
       </c>
       <c r="T65" s="19" t="n">
-        <f aca="false">IF(T56&gt;0,T$3,999)</f>
+        <f aca="false">IF(MIN(T56:$BJ56)&gt;0,T$3,999)</f>
         <v>999</v>
       </c>
       <c r="U65" s="19" t="n">
-        <f aca="false">IF(U56&gt;0,U$3,999)</f>
+        <f aca="false">IF(MIN(U56:$BJ56)&gt;0,U$3,999)</f>
         <v>999</v>
       </c>
       <c r="V65" s="19" t="n">
-        <f aca="false">IF(V56&gt;0,V$3,999)</f>
+        <f aca="false">IF(MIN(V56:$BJ56)&gt;0,V$3,999)</f>
         <v>999</v>
       </c>
       <c r="W65" s="19" t="n">
-        <f aca="false">IF(W56&gt;0,W$3,999)</f>
+        <f aca="false">IF(MIN(W56:$BJ56)&gt;0,W$3,999)</f>
         <v>999</v>
       </c>
       <c r="X65" s="19" t="n">
-        <f aca="false">IF(X56&gt;0,X$3,999)</f>
+        <f aca="false">IF(MIN(X56:$BJ56)&gt;0,X$3,999)</f>
         <v>999</v>
       </c>
       <c r="Y65" s="19" t="n">
-        <f aca="false">IF(Y56&gt;0,Y$3,999)</f>
+        <f aca="false">IF(MIN(Y56:$BJ56)&gt;0,Y$3,999)</f>
         <v>999</v>
       </c>
       <c r="Z65" s="19" t="n">
-        <f aca="false">IF(Z56&gt;0,Z$3,999)</f>
+        <f aca="false">IF(MIN(Z56:$BJ56)&gt;0,Z$3,999)</f>
         <v>999</v>
       </c>
       <c r="AA65" s="19" t="n">
-        <f aca="false">IF(AA56&gt;0,AA$3,999)</f>
+        <f aca="false">IF(MIN(AA56:$BJ56)&gt;0,AA$3,999)</f>
         <v>999</v>
       </c>
       <c r="AB65" s="19" t="n">
-        <f aca="false">IF(AB56&gt;0,AB$3,999)</f>
+        <f aca="false">IF(MIN(AB56:$BJ56)&gt;0,AB$3,999)</f>
         <v>999</v>
       </c>
       <c r="AC65" s="19" t="n">
-        <f aca="false">IF(AC56&gt;0,AC$3,999)</f>
+        <f aca="false">IF(MIN(AC56:$BJ56)&gt;0,AC$3,999)</f>
         <v>999</v>
       </c>
       <c r="AD65" s="19" t="n">
-        <f aca="false">IF(AD56&gt;0,AD$3,999)</f>
+        <f aca="false">IF(MIN(AD56:$BJ56)&gt;0,AD$3,999)</f>
         <v>999</v>
       </c>
       <c r="AE65" s="19" t="n">
-        <f aca="false">IF(AE56&gt;0,AE$3,999)</f>
+        <f aca="false">IF(MIN(AE56:$BJ56)&gt;0,AE$3,999)</f>
         <v>999</v>
       </c>
       <c r="AF65" s="19" t="n">
-        <f aca="false">IF(AF56&gt;0,AF$3,999)</f>
+        <f aca="false">IF(MIN(AF56:$BJ56)&gt;0,AF$3,999)</f>
         <v>999</v>
       </c>
       <c r="AG65" s="19" t="n">
-        <f aca="false">IF(AG56&gt;0,AG$3,999)</f>
+        <f aca="false">IF(MIN(AG56:$BJ56)&gt;0,AG$3,999)</f>
         <v>999</v>
       </c>
       <c r="AH65" s="19" t="n">
-        <f aca="false">IF(AH56&gt;0,AH$3,999)</f>
+        <f aca="false">IF(MIN(AH56:$BJ56)&gt;0,AH$3,999)</f>
         <v>999</v>
       </c>
       <c r="AI65" s="19" t="n">
-        <f aca="false">IF(AI56&gt;0,AI$3,999)</f>
+        <f aca="false">IF(MIN(AI56:$BJ56)&gt;0,AI$3,999)</f>
         <v>999</v>
       </c>
       <c r="AJ65" s="19" t="n">
-        <f aca="false">IF(AJ56&gt;0,AJ$3,999)</f>
+        <f aca="false">IF(MIN(AJ56:$BJ56)&gt;0,AJ$3,999)</f>
         <v>999</v>
       </c>
       <c r="AK65" s="19" t="n">
-        <f aca="false">IF(AK56&gt;0,AK$3,999)</f>
+        <f aca="false">IF(MIN(AK56:$BJ56)&gt;0,AK$3,999)</f>
         <v>999</v>
       </c>
       <c r="AL65" s="19" t="n">
-        <f aca="false">IF(AL56&gt;0,AL$3,999)</f>
+        <f aca="false">IF(MIN(AL56:$BJ56)&gt;0,AL$3,999)</f>
         <v>999</v>
       </c>
       <c r="AM65" s="19" t="n">
-        <f aca="false">IF(AM56&gt;0,AM$3,999)</f>
+        <f aca="false">IF(MIN(AM56:$BJ56)&gt;0,AM$3,999)</f>
         <v>999</v>
       </c>
       <c r="AN65" s="19" t="n">
-        <f aca="false">IF(AN56&gt;0,AN$3,999)</f>
+        <f aca="false">IF(MIN(AN56:$BJ56)&gt;0,AN$3,999)</f>
         <v>999</v>
       </c>
       <c r="AO65" s="19" t="n">
-        <f aca="false">IF(AO56&gt;0,AO$3,999)</f>
+        <f aca="false">IF(MIN(AO56:$BJ56)&gt;0,AO$3,999)</f>
         <v>999</v>
       </c>
       <c r="AP65" s="19" t="n">
-        <f aca="false">IF(AP56&gt;0,AP$3,999)</f>
+        <f aca="false">IF(MIN(AP56:$BJ56)&gt;0,AP$3,999)</f>
         <v>999</v>
       </c>
       <c r="AQ65" s="19" t="n">
-        <f aca="false">IF(AQ56&gt;0,AQ$3,999)</f>
+        <f aca="false">IF(MIN(AQ56:$BJ56)&gt;0,AQ$3,999)</f>
         <v>999</v>
       </c>
       <c r="AR65" s="19" t="n">
-        <f aca="false">IF(AR56&gt;0,AR$3,999)</f>
+        <f aca="false">IF(MIN(AR56:$BJ56)&gt;0,AR$3,999)</f>
         <v>999</v>
       </c>
       <c r="AS65" s="19" t="n">
-        <f aca="false">IF(AS56&gt;0,AS$3,999)</f>
+        <f aca="false">IF(MIN(AS56:$BJ56)&gt;0,AS$3,999)</f>
         <v>999</v>
       </c>
       <c r="AT65" s="19" t="n">
-        <f aca="false">IF(AT56&gt;0,AT$3,999)</f>
+        <f aca="false">IF(MIN(AT56:$BJ56)&gt;0,AT$3,999)</f>
         <v>999</v>
       </c>
       <c r="AU65" s="19" t="n">
-        <f aca="false">IF(AU56&gt;0,AU$3,999)</f>
+        <f aca="false">IF(MIN(AU56:$BJ56)&gt;0,AU$3,999)</f>
         <v>999</v>
       </c>
       <c r="AV65" s="19" t="n">
-        <f aca="false">IF(AV56&gt;0,AV$3,999)</f>
-        <v>46</v>
+        <f aca="false">IF(MIN(AV56:$BJ56)&gt;0,AV$3,999)</f>
+        <v>999</v>
       </c>
       <c r="AW65" s="19" t="n">
-        <f aca="false">IF(AW56&gt;0,AW$3,999)</f>
-        <v>47</v>
+        <f aca="false">IF(MIN(AW56:$BJ56)&gt;0,AW$3,999)</f>
+        <v>999</v>
       </c>
       <c r="AX65" s="19" t="n">
-        <f aca="false">IF(AX56&gt;0,AX$3,999)</f>
-        <v>48</v>
+        <f aca="false">IF(MIN(AX56:$BJ56)&gt;0,AX$3,999)</f>
+        <v>999</v>
       </c>
       <c r="AY65" s="19" t="n">
-        <f aca="false">IF(AY56&gt;0,AY$3,999)</f>
+        <f aca="false">IF(MIN(AY56:$BJ56)&gt;0,AY$3,999)</f>
         <v>999</v>
       </c>
       <c r="AZ65" s="19" t="n">
-        <f aca="false">IF(AZ56&gt;0,AZ$3,999)</f>
+        <f aca="false">IF(MIN(AZ56:$BJ56)&gt;0,AZ$3,999)</f>
         <v>50</v>
       </c>
       <c r="BA65" s="19" t="n">
-        <f aca="false">IF(BA56&gt;0,BA$3,999)</f>
+        <f aca="false">IF(MIN(BA56:$BJ56)&gt;0,BA$3,999)</f>
         <v>51</v>
       </c>
       <c r="BB65" s="19" t="n">
-        <f aca="false">IF(BB56&gt;0,BB$3,999)</f>
+        <f aca="false">IF(MIN(BB56:$BJ56)&gt;0,BB$3,999)</f>
         <v>52</v>
       </c>
       <c r="BC65" s="19" t="n">
-        <f aca="false">IF(BC56&gt;0,BC$3,999)</f>
+        <f aca="false">IF(MIN(BC56:$BJ56)&gt;0,BC$3,999)</f>
         <v>53</v>
       </c>
       <c r="BD65" s="19" t="n">
-        <f aca="false">IF(BD56&gt;0,BD$3,999)</f>
+        <f aca="false">IF(MIN(BD56:$BJ56)&gt;0,BD$3,999)</f>
         <v>54</v>
       </c>
       <c r="BE65" s="19" t="n">
-        <f aca="false">IF(BE56&gt;0,BE$3,999)</f>
+        <f aca="false">IF(MIN(BE56:$BJ56)&gt;0,BE$3,999)</f>
         <v>55</v>
       </c>
       <c r="BF65" s="19" t="n">
-        <f aca="false">IF(BF56&gt;0,BF$3,999)</f>
+        <f aca="false">IF(MIN(BF56:$BJ56)&gt;0,BF$3,999)</f>
         <v>56</v>
       </c>
       <c r="BG65" s="19" t="n">
-        <f aca="false">IF(BG56&gt;0,BG$3,999)</f>
+        <f aca="false">IF(MIN(BG56:$BJ56)&gt;0,BG$3,999)</f>
         <v>57</v>
       </c>
       <c r="BH65" s="19" t="n">
-        <f aca="false">IF(BH56&gt;0,BH$3,999)</f>
+        <f aca="false">IF(MIN(BH56:$BJ56)&gt;0,BH$3,999)</f>
         <v>58</v>
       </c>
       <c r="BI65" s="19" t="n">
-        <f aca="false">IF(BI56&gt;0,BI$3,999)</f>
+        <f aca="false">IF(MIN(BI56:$BJ56)&gt;0,BI$3,999)</f>
         <v>59</v>
       </c>
       <c r="BJ65" s="19" t="n">
-        <f aca="false">IF(BJ56&gt;0,BJ$3,999)</f>
+        <f aca="false">IF(MIN(BJ56:$BJ56)&gt;0,BJ$3,999)</f>
         <v>60</v>
       </c>
     </row>
@@ -32074,243 +32074,243 @@
         <v>264</v>
       </c>
       <c r="C65" s="19" t="n">
-        <f aca="false">IF(C56&gt;0,C$3,999)</f>
+        <f aca="false">IF(MIN(C56:$BJ56)&gt;0,C$3,999)</f>
         <v>999</v>
       </c>
       <c r="D65" s="19" t="n">
-        <f aca="false">IF(D56&gt;0,D$3,999)</f>
+        <f aca="false">IF(MIN(D56:$BJ56)&gt;0,D$3,999)</f>
         <v>999</v>
       </c>
       <c r="E65" s="19" t="n">
-        <f aca="false">IF(E56&gt;0,E$3,999)</f>
+        <f aca="false">IF(MIN(E56:$BJ56)&gt;0,E$3,999)</f>
         <v>999</v>
       </c>
       <c r="F65" s="19" t="n">
-        <f aca="false">IF(F56&gt;0,F$3,999)</f>
+        <f aca="false">IF(MIN(F56:$BJ56)&gt;0,F$3,999)</f>
         <v>999</v>
       </c>
       <c r="G65" s="19" t="n">
-        <f aca="false">IF(G56&gt;0,G$3,999)</f>
+        <f aca="false">IF(MIN(G56:$BJ56)&gt;0,G$3,999)</f>
         <v>999</v>
       </c>
       <c r="H65" s="19" t="n">
-        <f aca="false">IF(H56&gt;0,H$3,999)</f>
+        <f aca="false">IF(MIN(H56:$BJ56)&gt;0,H$3,999)</f>
         <v>999</v>
       </c>
       <c r="I65" s="19" t="n">
-        <f aca="false">IF(I56&gt;0,I$3,999)</f>
+        <f aca="false">IF(MIN(I56:$BJ56)&gt;0,I$3,999)</f>
         <v>999</v>
       </c>
       <c r="J65" s="19" t="n">
-        <f aca="false">IF(J56&gt;0,J$3,999)</f>
+        <f aca="false">IF(MIN(J56:$BJ56)&gt;0,J$3,999)</f>
         <v>999</v>
       </c>
       <c r="K65" s="19" t="n">
-        <f aca="false">IF(K56&gt;0,K$3,999)</f>
+        <f aca="false">IF(MIN(K56:$BJ56)&gt;0,K$3,999)</f>
         <v>999</v>
       </c>
       <c r="L65" s="19" t="n">
-        <f aca="false">IF(L56&gt;0,L$3,999)</f>
+        <f aca="false">IF(MIN(L56:$BJ56)&gt;0,L$3,999)</f>
         <v>999</v>
       </c>
       <c r="M65" s="19" t="n">
-        <f aca="false">IF(M56&gt;0,M$3,999)</f>
+        <f aca="false">IF(MIN(M56:$BJ56)&gt;0,M$3,999)</f>
         <v>999</v>
       </c>
       <c r="N65" s="19" t="n">
-        <f aca="false">IF(N56&gt;0,N$3,999)</f>
+        <f aca="false">IF(MIN(N56:$BJ56)&gt;0,N$3,999)</f>
         <v>999</v>
       </c>
       <c r="O65" s="19" t="n">
-        <f aca="false">IF(O56&gt;0,O$3,999)</f>
+        <f aca="false">IF(MIN(O56:$BJ56)&gt;0,O$3,999)</f>
         <v>999</v>
       </c>
       <c r="P65" s="19" t="n">
-        <f aca="false">IF(P56&gt;0,P$3,999)</f>
+        <f aca="false">IF(MIN(P56:$BJ56)&gt;0,P$3,999)</f>
         <v>999</v>
       </c>
       <c r="Q65" s="19" t="n">
-        <f aca="false">IF(Q56&gt;0,Q$3,999)</f>
+        <f aca="false">IF(MIN(Q56:$BJ56)&gt;0,Q$3,999)</f>
         <v>999</v>
       </c>
       <c r="R65" s="19" t="n">
-        <f aca="false">IF(R56&gt;0,R$3,999)</f>
+        <f aca="false">IF(MIN(R56:$BJ56)&gt;0,R$3,999)</f>
         <v>999</v>
       </c>
       <c r="S65" s="19" t="n">
-        <f aca="false">IF(S56&gt;0,S$3,999)</f>
+        <f aca="false">IF(MIN(S56:$BJ56)&gt;0,S$3,999)</f>
         <v>999</v>
       </c>
       <c r="T65" s="19" t="n">
-        <f aca="false">IF(T56&gt;0,T$3,999)</f>
+        <f aca="false">IF(MIN(T56:$BJ56)&gt;0,T$3,999)</f>
         <v>999</v>
       </c>
       <c r="U65" s="19" t="n">
-        <f aca="false">IF(U56&gt;0,U$3,999)</f>
+        <f aca="false">IF(MIN(U56:$BJ56)&gt;0,U$3,999)</f>
         <v>999</v>
       </c>
       <c r="V65" s="19" t="n">
-        <f aca="false">IF(V56&gt;0,V$3,999)</f>
+        <f aca="false">IF(MIN(V56:$BJ56)&gt;0,V$3,999)</f>
         <v>999</v>
       </c>
       <c r="W65" s="19" t="n">
-        <f aca="false">IF(W56&gt;0,W$3,999)</f>
+        <f aca="false">IF(MIN(W56:$BJ56)&gt;0,W$3,999)</f>
         <v>999</v>
       </c>
       <c r="X65" s="19" t="n">
-        <f aca="false">IF(X56&gt;0,X$3,999)</f>
+        <f aca="false">IF(MIN(X56:$BJ56)&gt;0,X$3,999)</f>
         <v>999</v>
       </c>
       <c r="Y65" s="19" t="n">
-        <f aca="false">IF(Y56&gt;0,Y$3,999)</f>
+        <f aca="false">IF(MIN(Y56:$BJ56)&gt;0,Y$3,999)</f>
         <v>999</v>
       </c>
       <c r="Z65" s="19" t="n">
-        <f aca="false">IF(Z56&gt;0,Z$3,999)</f>
+        <f aca="false">IF(MIN(Z56:$BJ56)&gt;0,Z$3,999)</f>
         <v>999</v>
       </c>
       <c r="AA65" s="19" t="n">
-        <f aca="false">IF(AA56&gt;0,AA$3,999)</f>
+        <f aca="false">IF(MIN(AA56:$BJ56)&gt;0,AA$3,999)</f>
         <v>999</v>
       </c>
       <c r="AB65" s="19" t="n">
-        <f aca="false">IF(AB56&gt;0,AB$3,999)</f>
+        <f aca="false">IF(MIN(AB56:$BJ56)&gt;0,AB$3,999)</f>
         <v>999</v>
       </c>
       <c r="AC65" s="19" t="n">
-        <f aca="false">IF(AC56&gt;0,AC$3,999)</f>
+        <f aca="false">IF(MIN(AC56:$BJ56)&gt;0,AC$3,999)</f>
         <v>999</v>
       </c>
       <c r="AD65" s="19" t="n">
-        <f aca="false">IF(AD56&gt;0,AD$3,999)</f>
+        <f aca="false">IF(MIN(AD56:$BJ56)&gt;0,AD$3,999)</f>
         <v>999</v>
       </c>
       <c r="AE65" s="19" t="n">
-        <f aca="false">IF(AE56&gt;0,AE$3,999)</f>
+        <f aca="false">IF(MIN(AE56:$BJ56)&gt;0,AE$3,999)</f>
         <v>999</v>
       </c>
       <c r="AF65" s="19" t="n">
-        <f aca="false">IF(AF56&gt;0,AF$3,999)</f>
+        <f aca="false">IF(MIN(AF56:$BJ56)&gt;0,AF$3,999)</f>
         <v>30</v>
       </c>
       <c r="AG65" s="19" t="n">
-        <f aca="false">IF(AG56&gt;0,AG$3,999)</f>
+        <f aca="false">IF(MIN(AG56:$BJ56)&gt;0,AG$3,999)</f>
         <v>31</v>
       </c>
       <c r="AH65" s="19" t="n">
-        <f aca="false">IF(AH56&gt;0,AH$3,999)</f>
+        <f aca="false">IF(MIN(AH56:$BJ56)&gt;0,AH$3,999)</f>
         <v>32</v>
       </c>
       <c r="AI65" s="19" t="n">
-        <f aca="false">IF(AI56&gt;0,AI$3,999)</f>
+        <f aca="false">IF(MIN(AI56:$BJ56)&gt;0,AI$3,999)</f>
         <v>33</v>
       </c>
       <c r="AJ65" s="19" t="n">
-        <f aca="false">IF(AJ56&gt;0,AJ$3,999)</f>
+        <f aca="false">IF(MIN(AJ56:$BJ56)&gt;0,AJ$3,999)</f>
         <v>34</v>
       </c>
       <c r="AK65" s="19" t="n">
-        <f aca="false">IF(AK56&gt;0,AK$3,999)</f>
+        <f aca="false">IF(MIN(AK56:$BJ56)&gt;0,AK$3,999)</f>
         <v>35</v>
       </c>
       <c r="AL65" s="19" t="n">
-        <f aca="false">IF(AL56&gt;0,AL$3,999)</f>
+        <f aca="false">IF(MIN(AL56:$BJ56)&gt;0,AL$3,999)</f>
         <v>36</v>
       </c>
       <c r="AM65" s="19" t="n">
-        <f aca="false">IF(AM56&gt;0,AM$3,999)</f>
+        <f aca="false">IF(MIN(AM56:$BJ56)&gt;0,AM$3,999)</f>
         <v>37</v>
       </c>
       <c r="AN65" s="19" t="n">
-        <f aca="false">IF(AN56&gt;0,AN$3,999)</f>
+        <f aca="false">IF(MIN(AN56:$BJ56)&gt;0,AN$3,999)</f>
         <v>38</v>
       </c>
       <c r="AO65" s="19" t="n">
-        <f aca="false">IF(AO56&gt;0,AO$3,999)</f>
+        <f aca="false">IF(MIN(AO56:$BJ56)&gt;0,AO$3,999)</f>
         <v>39</v>
       </c>
       <c r="AP65" s="19" t="n">
-        <f aca="false">IF(AP56&gt;0,AP$3,999)</f>
+        <f aca="false">IF(MIN(AP56:$BJ56)&gt;0,AP$3,999)</f>
         <v>40</v>
       </c>
       <c r="AQ65" s="19" t="n">
-        <f aca="false">IF(AQ56&gt;0,AQ$3,999)</f>
+        <f aca="false">IF(MIN(AQ56:$BJ56)&gt;0,AQ$3,999)</f>
         <v>41</v>
       </c>
       <c r="AR65" s="19" t="n">
-        <f aca="false">IF(AR56&gt;0,AR$3,999)</f>
+        <f aca="false">IF(MIN(AR56:$BJ56)&gt;0,AR$3,999)</f>
         <v>42</v>
       </c>
       <c r="AS65" s="19" t="n">
-        <f aca="false">IF(AS56&gt;0,AS$3,999)</f>
+        <f aca="false">IF(MIN(AS56:$BJ56)&gt;0,AS$3,999)</f>
         <v>43</v>
       </c>
       <c r="AT65" s="19" t="n">
-        <f aca="false">IF(AT56&gt;0,AT$3,999)</f>
+        <f aca="false">IF(MIN(AT56:$BJ56)&gt;0,AT$3,999)</f>
         <v>44</v>
       </c>
       <c r="AU65" s="19" t="n">
-        <f aca="false">IF(AU56&gt;0,AU$3,999)</f>
+        <f aca="false">IF(MIN(AU56:$BJ56)&gt;0,AU$3,999)</f>
         <v>45</v>
       </c>
       <c r="AV65" s="19" t="n">
-        <f aca="false">IF(AV56&gt;0,AV$3,999)</f>
+        <f aca="false">IF(MIN(AV56:$BJ56)&gt;0,AV$3,999)</f>
         <v>46</v>
       </c>
       <c r="AW65" s="19" t="n">
-        <f aca="false">IF(AW56&gt;0,AW$3,999)</f>
+        <f aca="false">IF(MIN(AW56:$BJ56)&gt;0,AW$3,999)</f>
         <v>47</v>
       </c>
       <c r="AX65" s="19" t="n">
-        <f aca="false">IF(AX56&gt;0,AX$3,999)</f>
+        <f aca="false">IF(MIN(AX56:$BJ56)&gt;0,AX$3,999)</f>
         <v>48</v>
       </c>
       <c r="AY65" s="19" t="n">
-        <f aca="false">IF(AY56&gt;0,AY$3,999)</f>
+        <f aca="false">IF(MIN(AY56:$BJ56)&gt;0,AY$3,999)</f>
         <v>49</v>
       </c>
       <c r="AZ65" s="19" t="n">
-        <f aca="false">IF(AZ56&gt;0,AZ$3,999)</f>
+        <f aca="false">IF(MIN(AZ56:$BJ56)&gt;0,AZ$3,999)</f>
         <v>50</v>
       </c>
       <c r="BA65" s="19" t="n">
-        <f aca="false">IF(BA56&gt;0,BA$3,999)</f>
+        <f aca="false">IF(MIN(BA56:$BJ56)&gt;0,BA$3,999)</f>
         <v>51</v>
       </c>
       <c r="BB65" s="19" t="n">
-        <f aca="false">IF(BB56&gt;0,BB$3,999)</f>
+        <f aca="false">IF(MIN(BB56:$BJ56)&gt;0,BB$3,999)</f>
         <v>52</v>
       </c>
       <c r="BC65" s="19" t="n">
-        <f aca="false">IF(BC56&gt;0,BC$3,999)</f>
+        <f aca="false">IF(MIN(BC56:$BJ56)&gt;0,BC$3,999)</f>
         <v>53</v>
       </c>
       <c r="BD65" s="19" t="n">
-        <f aca="false">IF(BD56&gt;0,BD$3,999)</f>
+        <f aca="false">IF(MIN(BD56:$BJ56)&gt;0,BD$3,999)</f>
         <v>54</v>
       </c>
       <c r="BE65" s="19" t="n">
-        <f aca="false">IF(BE56&gt;0,BE$3,999)</f>
+        <f aca="false">IF(MIN(BE56:$BJ56)&gt;0,BE$3,999)</f>
         <v>55</v>
       </c>
       <c r="BF65" s="19" t="n">
-        <f aca="false">IF(BF56&gt;0,BF$3,999)</f>
+        <f aca="false">IF(MIN(BF56:$BJ56)&gt;0,BF$3,999)</f>
         <v>56</v>
       </c>
       <c r="BG65" s="19" t="n">
-        <f aca="false">IF(BG56&gt;0,BG$3,999)</f>
+        <f aca="false">IF(MIN(BG56:$BJ56)&gt;0,BG$3,999)</f>
         <v>57</v>
       </c>
       <c r="BH65" s="19" t="n">
-        <f aca="false">IF(BH56&gt;0,BH$3,999)</f>
+        <f aca="false">IF(MIN(BH56:$BJ56)&gt;0,BH$3,999)</f>
         <v>58</v>
       </c>
       <c r="BI65" s="19" t="n">
-        <f aca="false">IF(BI56&gt;0,BI$3,999)</f>
+        <f aca="false">IF(MIN(BI56:$BJ56)&gt;0,BI$3,999)</f>
         <v>59</v>
       </c>
       <c r="BJ65" s="19" t="n">
-        <f aca="false">IF(BJ56&gt;0,BJ$3,999)</f>
+        <f aca="false">IF(MIN(BJ56:$BJ56)&gt;0,BJ$3,999)</f>
         <v>60</v>
       </c>
     </row>
@@ -45626,243 +45626,243 @@
         <v>264</v>
       </c>
       <c r="C65" s="19" t="n">
-        <f aca="false">IF(C56&gt;0,C$3,999)</f>
+        <f aca="false">IF(MIN(C56:$BJ56)&gt;0,C$3,999)</f>
         <v>999</v>
       </c>
       <c r="D65" s="19" t="n">
-        <f aca="false">IF(D56&gt;0,D$3,999)</f>
+        <f aca="false">IF(MIN(D56:$BJ56)&gt;0,D$3,999)</f>
         <v>999</v>
       </c>
       <c r="E65" s="19" t="n">
-        <f aca="false">IF(E56&gt;0,E$3,999)</f>
+        <f aca="false">IF(MIN(E56:$BJ56)&gt;0,E$3,999)</f>
         <v>999</v>
       </c>
       <c r="F65" s="19" t="n">
-        <f aca="false">IF(F56&gt;0,F$3,999)</f>
+        <f aca="false">IF(MIN(F56:$BJ56)&gt;0,F$3,999)</f>
         <v>999</v>
       </c>
       <c r="G65" s="19" t="n">
-        <f aca="false">IF(G56&gt;0,G$3,999)</f>
+        <f aca="false">IF(MIN(G56:$BJ56)&gt;0,G$3,999)</f>
         <v>999</v>
       </c>
       <c r="H65" s="19" t="n">
-        <f aca="false">IF(H56&gt;0,H$3,999)</f>
+        <f aca="false">IF(MIN(H56:$BJ56)&gt;0,H$3,999)</f>
         <v>999</v>
       </c>
       <c r="I65" s="19" t="n">
-        <f aca="false">IF(I56&gt;0,I$3,999)</f>
+        <f aca="false">IF(MIN(I56:$BJ56)&gt;0,I$3,999)</f>
         <v>999</v>
       </c>
       <c r="J65" s="19" t="n">
-        <f aca="false">IF(J56&gt;0,J$3,999)</f>
+        <f aca="false">IF(MIN(J56:$BJ56)&gt;0,J$3,999)</f>
         <v>999</v>
       </c>
       <c r="K65" s="19" t="n">
-        <f aca="false">IF(K56&gt;0,K$3,999)</f>
+        <f aca="false">IF(MIN(K56:$BJ56)&gt;0,K$3,999)</f>
         <v>999</v>
       </c>
       <c r="L65" s="19" t="n">
-        <f aca="false">IF(L56&gt;0,L$3,999)</f>
+        <f aca="false">IF(MIN(L56:$BJ56)&gt;0,L$3,999)</f>
         <v>999</v>
       </c>
       <c r="M65" s="19" t="n">
-        <f aca="false">IF(M56&gt;0,M$3,999)</f>
+        <f aca="false">IF(MIN(M56:$BJ56)&gt;0,M$3,999)</f>
         <v>999</v>
       </c>
       <c r="N65" s="19" t="n">
-        <f aca="false">IF(N56&gt;0,N$3,999)</f>
+        <f aca="false">IF(MIN(N56:$BJ56)&gt;0,N$3,999)</f>
         <v>999</v>
       </c>
       <c r="O65" s="19" t="n">
-        <f aca="false">IF(O56&gt;0,O$3,999)</f>
+        <f aca="false">IF(MIN(O56:$BJ56)&gt;0,O$3,999)</f>
         <v>999</v>
       </c>
       <c r="P65" s="19" t="n">
-        <f aca="false">IF(P56&gt;0,P$3,999)</f>
+        <f aca="false">IF(MIN(P56:$BJ56)&gt;0,P$3,999)</f>
         <v>999</v>
       </c>
       <c r="Q65" s="19" t="n">
-        <f aca="false">IF(Q56&gt;0,Q$3,999)</f>
+        <f aca="false">IF(MIN(Q56:$BJ56)&gt;0,Q$3,999)</f>
         <v>999</v>
       </c>
       <c r="R65" s="19" t="n">
-        <f aca="false">IF(R56&gt;0,R$3,999)</f>
+        <f aca="false">IF(MIN(R56:$BJ56)&gt;0,R$3,999)</f>
         <v>999</v>
       </c>
       <c r="S65" s="19" t="n">
-        <f aca="false">IF(S56&gt;0,S$3,999)</f>
+        <f aca="false">IF(MIN(S56:$BJ56)&gt;0,S$3,999)</f>
         <v>999</v>
       </c>
       <c r="T65" s="19" t="n">
-        <f aca="false">IF(T56&gt;0,T$3,999)</f>
+        <f aca="false">IF(MIN(T56:$BJ56)&gt;0,T$3,999)</f>
         <v>999</v>
       </c>
       <c r="U65" s="19" t="n">
-        <f aca="false">IF(U56&gt;0,U$3,999)</f>
+        <f aca="false">IF(MIN(U56:$BJ56)&gt;0,U$3,999)</f>
         <v>999</v>
       </c>
       <c r="V65" s="19" t="n">
-        <f aca="false">IF(V56&gt;0,V$3,999)</f>
+        <f aca="false">IF(MIN(V56:$BJ56)&gt;0,V$3,999)</f>
         <v>999</v>
       </c>
       <c r="W65" s="19" t="n">
-        <f aca="false">IF(W56&gt;0,W$3,999)</f>
-        <v>21</v>
+        <f aca="false">IF(MIN(W56:$BJ56)&gt;0,W$3,999)</f>
+        <v>999</v>
       </c>
       <c r="X65" s="19" t="n">
-        <f aca="false">IF(X56&gt;0,X$3,999)</f>
-        <v>22</v>
+        <f aca="false">IF(MIN(X56:$BJ56)&gt;0,X$3,999)</f>
+        <v>999</v>
       </c>
       <c r="Y65" s="19" t="n">
-        <f aca="false">IF(Y56&gt;0,Y$3,999)</f>
-        <v>23</v>
+        <f aca="false">IF(MIN(Y56:$BJ56)&gt;0,Y$3,999)</f>
+        <v>999</v>
       </c>
       <c r="Z65" s="19" t="n">
-        <f aca="false">IF(Z56&gt;0,Z$3,999)</f>
-        <v>24</v>
+        <f aca="false">IF(MIN(Z56:$BJ56)&gt;0,Z$3,999)</f>
+        <v>999</v>
       </c>
       <c r="AA65" s="19" t="n">
-        <f aca="false">IF(AA56&gt;0,AA$3,999)</f>
+        <f aca="false">IF(MIN(AA56:$BJ56)&gt;0,AA$3,999)</f>
         <v>999</v>
       </c>
       <c r="AB65" s="19" t="n">
-        <f aca="false">IF(AB56&gt;0,AB$3,999)</f>
+        <f aca="false">IF(MIN(AB56:$BJ56)&gt;0,AB$3,999)</f>
         <v>999</v>
       </c>
       <c r="AC65" s="19" t="n">
-        <f aca="false">IF(AC56&gt;0,AC$3,999)</f>
+        <f aca="false">IF(MIN(AC56:$BJ56)&gt;0,AC$3,999)</f>
         <v>27</v>
       </c>
       <c r="AD65" s="19" t="n">
-        <f aca="false">IF(AD56&gt;0,AD$3,999)</f>
+        <f aca="false">IF(MIN(AD56:$BJ56)&gt;0,AD$3,999)</f>
         <v>28</v>
       </c>
       <c r="AE65" s="19" t="n">
-        <f aca="false">IF(AE56&gt;0,AE$3,999)</f>
+        <f aca="false">IF(MIN(AE56:$BJ56)&gt;0,AE$3,999)</f>
         <v>29</v>
       </c>
       <c r="AF65" s="19" t="n">
-        <f aca="false">IF(AF56&gt;0,AF$3,999)</f>
+        <f aca="false">IF(MIN(AF56:$BJ56)&gt;0,AF$3,999)</f>
         <v>30</v>
       </c>
       <c r="AG65" s="19" t="n">
-        <f aca="false">IF(AG56&gt;0,AG$3,999)</f>
+        <f aca="false">IF(MIN(AG56:$BJ56)&gt;0,AG$3,999)</f>
         <v>31</v>
       </c>
       <c r="AH65" s="19" t="n">
-        <f aca="false">IF(AH56&gt;0,AH$3,999)</f>
+        <f aca="false">IF(MIN(AH56:$BJ56)&gt;0,AH$3,999)</f>
         <v>32</v>
       </c>
       <c r="AI65" s="19" t="n">
-        <f aca="false">IF(AI56&gt;0,AI$3,999)</f>
+        <f aca="false">IF(MIN(AI56:$BJ56)&gt;0,AI$3,999)</f>
         <v>33</v>
       </c>
       <c r="AJ65" s="19" t="n">
-        <f aca="false">IF(AJ56&gt;0,AJ$3,999)</f>
+        <f aca="false">IF(MIN(AJ56:$BJ56)&gt;0,AJ$3,999)</f>
         <v>34</v>
       </c>
       <c r="AK65" s="19" t="n">
-        <f aca="false">IF(AK56&gt;0,AK$3,999)</f>
+        <f aca="false">IF(MIN(AK56:$BJ56)&gt;0,AK$3,999)</f>
         <v>35</v>
       </c>
       <c r="AL65" s="19" t="n">
-        <f aca="false">IF(AL56&gt;0,AL$3,999)</f>
+        <f aca="false">IF(MIN(AL56:$BJ56)&gt;0,AL$3,999)</f>
         <v>36</v>
       </c>
       <c r="AM65" s="19" t="n">
-        <f aca="false">IF(AM56&gt;0,AM$3,999)</f>
+        <f aca="false">IF(MIN(AM56:$BJ56)&gt;0,AM$3,999)</f>
         <v>37</v>
       </c>
       <c r="AN65" s="19" t="n">
-        <f aca="false">IF(AN56&gt;0,AN$3,999)</f>
+        <f aca="false">IF(MIN(AN56:$BJ56)&gt;0,AN$3,999)</f>
         <v>38</v>
       </c>
       <c r="AO65" s="19" t="n">
-        <f aca="false">IF(AO56&gt;0,AO$3,999)</f>
+        <f aca="false">IF(MIN(AO56:$BJ56)&gt;0,AO$3,999)</f>
         <v>39</v>
       </c>
       <c r="AP65" s="19" t="n">
-        <f aca="false">IF(AP56&gt;0,AP$3,999)</f>
+        <f aca="false">IF(MIN(AP56:$BJ56)&gt;0,AP$3,999)</f>
         <v>40</v>
       </c>
       <c r="AQ65" s="19" t="n">
-        <f aca="false">IF(AQ56&gt;0,AQ$3,999)</f>
+        <f aca="false">IF(MIN(AQ56:$BJ56)&gt;0,AQ$3,999)</f>
         <v>41</v>
       </c>
       <c r="AR65" s="19" t="n">
-        <f aca="false">IF(AR56&gt;0,AR$3,999)</f>
+        <f aca="false">IF(MIN(AR56:$BJ56)&gt;0,AR$3,999)</f>
         <v>42</v>
       </c>
       <c r="AS65" s="19" t="n">
-        <f aca="false">IF(AS56&gt;0,AS$3,999)</f>
+        <f aca="false">IF(MIN(AS56:$BJ56)&gt;0,AS$3,999)</f>
         <v>43</v>
       </c>
       <c r="AT65" s="19" t="n">
-        <f aca="false">IF(AT56&gt;0,AT$3,999)</f>
+        <f aca="false">IF(MIN(AT56:$BJ56)&gt;0,AT$3,999)</f>
         <v>44</v>
       </c>
       <c r="AU65" s="19" t="n">
-        <f aca="false">IF(AU56&gt;0,AU$3,999)</f>
+        <f aca="false">IF(MIN(AU56:$BJ56)&gt;0,AU$3,999)</f>
         <v>45</v>
       </c>
       <c r="AV65" s="19" t="n">
-        <f aca="false">IF(AV56&gt;0,AV$3,999)</f>
+        <f aca="false">IF(MIN(AV56:$BJ56)&gt;0,AV$3,999)</f>
         <v>46</v>
       </c>
       <c r="AW65" s="19" t="n">
-        <f aca="false">IF(AW56&gt;0,AW$3,999)</f>
+        <f aca="false">IF(MIN(AW56:$BJ56)&gt;0,AW$3,999)</f>
         <v>47</v>
       </c>
       <c r="AX65" s="19" t="n">
-        <f aca="false">IF(AX56&gt;0,AX$3,999)</f>
+        <f aca="false">IF(MIN(AX56:$BJ56)&gt;0,AX$3,999)</f>
         <v>48</v>
       </c>
       <c r="AY65" s="19" t="n">
-        <f aca="false">IF(AY56&gt;0,AY$3,999)</f>
+        <f aca="false">IF(MIN(AY56:$BJ56)&gt;0,AY$3,999)</f>
         <v>49</v>
       </c>
       <c r="AZ65" s="19" t="n">
-        <f aca="false">IF(AZ56&gt;0,AZ$3,999)</f>
+        <f aca="false">IF(MIN(AZ56:$BJ56)&gt;0,AZ$3,999)</f>
         <v>50</v>
       </c>
       <c r="BA65" s="19" t="n">
-        <f aca="false">IF(BA56&gt;0,BA$3,999)</f>
+        <f aca="false">IF(MIN(BA56:$BJ56)&gt;0,BA$3,999)</f>
         <v>51</v>
       </c>
       <c r="BB65" s="19" t="n">
-        <f aca="false">IF(BB56&gt;0,BB$3,999)</f>
+        <f aca="false">IF(MIN(BB56:$BJ56)&gt;0,BB$3,999)</f>
         <v>52</v>
       </c>
       <c r="BC65" s="19" t="n">
-        <f aca="false">IF(BC56&gt;0,BC$3,999)</f>
+        <f aca="false">IF(MIN(BC56:$BJ56)&gt;0,BC$3,999)</f>
         <v>53</v>
       </c>
       <c r="BD65" s="19" t="n">
-        <f aca="false">IF(BD56&gt;0,BD$3,999)</f>
+        <f aca="false">IF(MIN(BD56:$BJ56)&gt;0,BD$3,999)</f>
         <v>54</v>
       </c>
       <c r="BE65" s="19" t="n">
-        <f aca="false">IF(BE56&gt;0,BE$3,999)</f>
+        <f aca="false">IF(MIN(BE56:$BJ56)&gt;0,BE$3,999)</f>
         <v>55</v>
       </c>
       <c r="BF65" s="19" t="n">
-        <f aca="false">IF(BF56&gt;0,BF$3,999)</f>
+        <f aca="false">IF(MIN(BF56:$BJ56)&gt;0,BF$3,999)</f>
         <v>56</v>
       </c>
       <c r="BG65" s="19" t="n">
-        <f aca="false">IF(BG56&gt;0,BG$3,999)</f>
+        <f aca="false">IF(MIN(BG56:$BJ56)&gt;0,BG$3,999)</f>
         <v>57</v>
       </c>
       <c r="BH65" s="19" t="n">
-        <f aca="false">IF(BH56&gt;0,BH$3,999)</f>
+        <f aca="false">IF(MIN(BH56:$BJ56)&gt;0,BH$3,999)</f>
         <v>58</v>
       </c>
       <c r="BI65" s="19" t="n">
-        <f aca="false">IF(BI56&gt;0,BI$3,999)</f>
+        <f aca="false">IF(MIN(BI56:$BJ56)&gt;0,BI$3,999)</f>
         <v>59</v>
       </c>
       <c r="BJ65" s="19" t="n">
-        <f aca="false">IF(BJ56&gt;0,BJ$3,999)</f>
+        <f aca="false">IF(MIN(BJ56:$BJ56)&gt;0,BJ$3,999)</f>
         <v>60</v>
       </c>
     </row>

</xml_diff>